<commit_message>
standardising output folder names in scripts 2 and 3, plus cosmetic changes to control files and code
</commit_message>
<xml_diff>
--- a/2_profile_generator/control_file_profile_generator.xlsx
+++ b/2_profile_generator/control_file_profile_generator.xlsx
@@ -1,23 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/MSR code repo/2_profile_generator/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_DDEDB4A8BED604FDB0E8A2ADE1532E5F302D5BA1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE0AEFD-B7F4-4455-9CF1-36869681E201}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="paths"/>
-    <sheet r:id="rId2" sheetId="2" name="configurations"/>
-    <sheet r:id="rId3" sheetId="3" name="parameters"/>
-    <sheet r:id="rId4" sheetId="4" name="datasets"/>
+    <sheet name="paths" sheetId="1" r:id="rId1"/>
+    <sheet name="configurations" sheetId="2" r:id="rId2"/>
+    <sheet name="parameters" sheetId="3" r:id="rId3"/>
+    <sheet name="datasets" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="55">
   <si>
     <t>datasets</t>
   </si>
@@ -258,18 +264,6 @@
     <t>paths</t>
   </si>
   <si>
-    <t>output_folder_msr_creator</t>
-  </si>
-  <si>
-    <t>C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\outputs\1_msr_creator</t>
-  </si>
-  <si>
-    <t>Folder path where msr creator ouputs are located.</t>
-  </si>
-  <si>
-    <t>input_datasets_folder</t>
-  </si>
-  <si>
     <t>C:\Users\mastt\OneDrive - VITO\Documents\21_WP1\RawData\model_supply_regions\workflow\inputs\2022 MSR Toolset Inputs</t>
   </si>
   <si>
@@ -279,21 +273,20 @@
     <t>output_folder</t>
   </si>
   <si>
-    <t>C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\outputs\2_profile_generator</t>
-  </si>
-  <si>
-    <t>output_folder_profile_generator</t>
-  </si>
-  <si>
-    <t>Folder path where profile generator ouputs are located.</t>
+    <t>input_folder_datasets</t>
+  </si>
+  <si>
+    <t>Folder path where outputs are located.</t>
+  </si>
+  <si>
+    <t>C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\outputs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -319,6 +312,21 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -348,115 +356,106 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C13" displayName="Table4" name="Table4" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:C13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:C3" totalsRowShown="0">
+  <autoFilter ref="A1:C3" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
-    <tableColumn name="datasets" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="paths"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C4" displayName="Table5" name="Table5" id="2" totalsRowShown="0">
-  <autoFilter ref="A1:C4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table1" displayName="Table1" ref="A1:C5" totalsRowShown="0">
+  <autoFilter ref="A1:C5" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="3">
-    <tableColumn name="parameters" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="configurations"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C5" displayName="Table1" name="Table1" id="3" totalsRowShown="0">
-  <autoFilter ref="A1:C5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A1:C4" totalsRowShown="0">
+  <autoFilter ref="A1:C4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
-    <tableColumn name="configurations" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="parameters"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C5" displayName="Table2" name="Table2" id="4" totalsRowShown="0">
-  <autoFilter ref="A1:C5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="A1:C13" totalsRowShown="0">
+  <autoFilter ref="A1:C13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn name="paths" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="datasets"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -465,10 +464,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -506,71 +505,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -598,7 +597,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -621,11 +620,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -634,13 +633,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -650,7 +649,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -659,7 +658,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -668,7 +667,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -676,10 +675,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -744,19 +743,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="5" width="36.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="58.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="52.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="36.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.81640625" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
@@ -767,46 +766,26 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="16"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -818,67 +797,67 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="6" width="48.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="60.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="48.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.81640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.7265625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>0</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="3">
+    <row r="3" spans="1:3" s="3" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <v>0</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="3">
+    <row r="4" spans="1:3" s="3" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="12">
         <v>1</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5" customFormat="1" s="3">
+    <row r="5" spans="1:3" s="3" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <v>0</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -894,55 +873,53 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="11" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="11.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>8784</v>
       </c>
-      <c r="C2" s="7"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="7" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>3000</v>
       </c>
-      <c r="C3" s="7"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="7" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="8">
         <v>100</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" t="s">
         <v>41</v>
       </c>
     </row>
@@ -955,19 +932,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="5" width="36.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="36.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="36.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="36.7265625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.7265625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -978,7 +954,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="2" spans="1:3" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -989,7 +965,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="3" spans="1:3" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -1000,7 +976,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="4" spans="1:3" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -1011,7 +987,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1022,7 +998,7 @@
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="6" spans="1:3" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
@@ -1033,7 +1009,7 @@
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="7" spans="1:3" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -1044,7 +1020,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
@@ -1055,7 +1031,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="9" spans="1:3" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>24</v>
       </c>
@@ -1066,7 +1042,7 @@
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="10" spans="1:3" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>27</v>
       </c>
@@ -1077,7 +1053,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="11" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
@@ -1086,7 +1062,7 @@
       </c>
       <c r="C11" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="12" spans="1:3" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
@@ -1097,7 +1073,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row r="13" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>35</v>
       </c>

</xml_diff>